<commit_message>
Sskx: update something (#2339)
* Sskx: update something

* Update sskx vorlage

* Update table reference

---------

Co-authored-by: eclipse-set-bot <set-bot@eclipse.org>
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskx_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskx_vorlage.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\PlanPro\docs\agate\PT_1_Tabellen\Excel-Vorlage\1.10.0.1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\SET\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D166EC3-7891-4048-BB5E-D05659B1AF54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8F5BD7-5BA9-43A1-97ED-3E489B87791E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" tabRatio="501" xr2:uid="{5D844E15-32D4-4E4F-AD6A-36EA8900B557}"/>
+    <workbookView xWindow="8595" yWindow="2475" windowWidth="28800" windowHeight="15345" tabRatio="501" xr2:uid="{5D844E15-32D4-4E4F-AD6A-36EA8900B557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sskx_Beispielbefüllung" sheetId="2" r:id="rId1"/>
@@ -129,9 +129,6 @@
 u. SO</t>
   </si>
   <si>
-    <t>Bezeichnung</t>
-  </si>
-  <si>
     <t>mm</t>
   </si>
   <si>
@@ -157,6 +154,9 @@
   </si>
   <si>
     <t>Gleis</t>
+  </si>
+  <si>
+    <t>Bezeichnung (Symbol)</t>
   </si>
 </sst>
 </file>
@@ -448,7 +448,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -519,53 +519,50 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1014,25 +1011,25 @@
       <c r="B2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="K2" s="30"/>
-      <c r="L2" s="30"/>
-      <c r="M2" s="31"/>
-      <c r="N2" s="29" t="s">
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="38"/>
+      <c r="N2" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="O2" s="30"/>
+      <c r="O2" s="37"/>
       <c r="P2" s="12" t="s">
         <v>18</v>
       </c>
@@ -1040,33 +1037,33 @@
     <row r="3" spans="1:16" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="4"/>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="28"/>
-      <c r="E3" s="25"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="32"/>
       <c r="F3" s="3" t="s">
         <v>20</v>
       </c>
       <c r="G3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" s="25"/>
-      <c r="J3" s="26" t="s">
+      <c r="H3" s="31" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="32"/>
+      <c r="J3" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="25"/>
-      <c r="L3" s="24" t="s">
+      <c r="K3" s="32"/>
+      <c r="L3" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="M3" s="27"/>
-      <c r="N3" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" s="27"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" s="34"/>
       <c r="P3" s="20"/>
     </row>
     <row r="4" spans="1:16" s="2" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1079,15 +1076,15 @@
         <v>25</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="8" t="s">
         <v>32</v>
-      </c>
-      <c r="I4" s="8" t="s">
-        <v>33</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>26</v>
@@ -1096,13 +1093,13 @@
         <v>27</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="M4" s="22" t="s">
         <v>28</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="O4" s="6" t="s">
         <v>27</v>
@@ -1117,923 +1114,573 @@
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J5" s="10"/>
       <c r="K5" s="11"/>
       <c r="L5" s="11"/>
       <c r="M5" s="23" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N5" s="10"/>
       <c r="O5" s="11"/>
       <c r="P5" s="19"/>
     </row>
     <row r="6" spans="1:16" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="39"/>
-      <c r="B6" s="33"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="35"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="37"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="37"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="37"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="38"/>
+      <c r="A6" s="30"/>
+      <c r="B6" s="25"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="27"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="M6" s="28"/>
+      <c r="P6" s="29"/>
     </row>
     <row r="7" spans="1:16" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="32"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="34"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="34"/>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
-      <c r="M7" s="37"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="34"/>
-      <c r="P7" s="38"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="25"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="27"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="M7" s="28"/>
+      <c r="P7" s="29"/>
     </row>
     <row r="8" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="32"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="34"/>
-      <c r="M8" s="37"/>
-      <c r="N8" s="34"/>
-      <c r="O8" s="34"/>
-      <c r="P8" s="38"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="25"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="27"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="M8" s="28"/>
+      <c r="P8" s="29"/>
     </row>
     <row r="9" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="32"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="37"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="37"/>
-      <c r="J9" s="34"/>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="34"/>
-      <c r="P9" s="38"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="25"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="27"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="M9" s="28"/>
+      <c r="P9" s="29"/>
     </row>
     <row r="10" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="32"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="36"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="37"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="37"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="38"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="25"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="M10" s="28"/>
+      <c r="P10" s="29"/>
     </row>
     <row r="11" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="32"/>
-      <c r="B11" s="33"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="36"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="37"/>
-      <c r="H11" s="37"/>
-      <c r="I11" s="37"/>
-      <c r="J11" s="34"/>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="37"/>
-      <c r="N11" s="34"/>
-      <c r="O11" s="34"/>
-      <c r="P11" s="38"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="25"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="27"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="M11" s="28"/>
+      <c r="P11" s="29"/>
     </row>
     <row r="12" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="32"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="34"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="36"/>
-      <c r="F12" s="34"/>
-      <c r="G12" s="37"/>
-      <c r="H12" s="37"/>
-      <c r="I12" s="37"/>
-      <c r="J12" s="34"/>
-      <c r="K12" s="34"/>
-      <c r="L12" s="34"/>
-      <c r="M12" s="37"/>
-      <c r="N12" s="34"/>
-      <c r="O12" s="34"/>
-      <c r="P12" s="38"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="25"/>
+      <c r="D12" s="26"/>
+      <c r="E12" s="27"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="M12" s="28"/>
+      <c r="P12" s="29"/>
     </row>
     <row r="13" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="34"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="34"/>
-      <c r="K13" s="34"/>
-      <c r="L13" s="34"/>
-      <c r="M13" s="37"/>
-      <c r="N13" s="34"/>
-      <c r="O13" s="34"/>
-      <c r="P13" s="38"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="25"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="27"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="M13" s="28"/>
+      <c r="P13" s="29"/>
     </row>
     <row r="14" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="32"/>
-      <c r="B14" s="33"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37"/>
-      <c r="I14" s="37"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="34"/>
-      <c r="M14" s="37"/>
-      <c r="N14" s="34"/>
-      <c r="O14" s="34"/>
-      <c r="P14" s="38"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="25"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="27"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="M14" s="28"/>
+      <c r="P14" s="29"/>
     </row>
     <row r="15" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="32"/>
-      <c r="B15" s="33"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="37"/>
-      <c r="H15" s="37"/>
-      <c r="I15" s="37"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="34"/>
-      <c r="L15" s="34"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="34"/>
-      <c r="O15" s="34"/>
-      <c r="P15" s="38"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="25"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="27"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="M15" s="28"/>
+      <c r="P15" s="29"/>
     </row>
     <row r="16" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="32"/>
-      <c r="B16" s="33"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="37"/>
-      <c r="H16" s="37"/>
-      <c r="I16" s="37"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
-      <c r="M16" s="37"/>
-      <c r="N16" s="34"/>
-      <c r="O16" s="34"/>
-      <c r="P16" s="38"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="25"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="27"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="M16" s="28"/>
+      <c r="P16" s="29"/>
     </row>
     <row r="17" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
-      <c r="B17" s="33"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="34"/>
-      <c r="G17" s="37"/>
-      <c r="H17" s="37"/>
-      <c r="I17" s="37"/>
-      <c r="J17" s="34"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="34"/>
-      <c r="M17" s="37"/>
-      <c r="N17" s="34"/>
-      <c r="O17" s="34"/>
-      <c r="P17" s="38"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="25"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="27"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="M17" s="28"/>
+      <c r="P17" s="29"/>
     </row>
     <row r="18" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="32"/>
-      <c r="B18" s="33"/>
-      <c r="C18" s="34"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="34"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="37"/>
-      <c r="I18" s="37"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="34"/>
-      <c r="O18" s="34"/>
-      <c r="P18" s="38"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="25"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="27"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="M18" s="28"/>
+      <c r="P18" s="29"/>
     </row>
     <row r="19" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="32"/>
-      <c r="B19" s="33"/>
-      <c r="C19" s="34"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="37"/>
-      <c r="I19" s="37"/>
-      <c r="J19" s="34"/>
-      <c r="K19" s="34"/>
-      <c r="L19" s="34"/>
-      <c r="M19" s="37"/>
-      <c r="N19" s="34"/>
-      <c r="O19" s="34"/>
-      <c r="P19" s="38"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="25"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="27"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="M19" s="28"/>
+      <c r="P19" s="29"/>
     </row>
     <row r="20" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="32"/>
-      <c r="B20" s="33"/>
-      <c r="C20" s="34"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="34"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="37"/>
-      <c r="I20" s="37"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
-      <c r="M20" s="37"/>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
-      <c r="P20" s="38"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="25"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="27"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="M20" s="28"/>
+      <c r="P20" s="29"/>
     </row>
     <row r="21" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="32"/>
-      <c r="B21" s="33"/>
-      <c r="C21" s="34"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="37"/>
-      <c r="H21" s="37"/>
-      <c r="I21" s="37"/>
-      <c r="J21" s="34"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="34"/>
-      <c r="M21" s="37"/>
-      <c r="N21" s="34"/>
-      <c r="O21" s="34"/>
-      <c r="P21" s="38"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="25"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="27"/>
+      <c r="G21" s="28"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="28"/>
+      <c r="M21" s="28"/>
+      <c r="P21" s="29"/>
     </row>
     <row r="22" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="32"/>
-      <c r="B22" s="33"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37"/>
-      <c r="I22" s="37"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="34"/>
-      <c r="M22" s="37"/>
-      <c r="N22" s="34"/>
-      <c r="O22" s="34"/>
-      <c r="P22" s="38"/>
+      <c r="A22" s="24"/>
+      <c r="B22" s="25"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="27"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="28"/>
+      <c r="I22" s="28"/>
+      <c r="M22" s="28"/>
+      <c r="P22" s="29"/>
     </row>
     <row r="23" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="32"/>
-      <c r="B23" s="33"/>
-      <c r="C23" s="34"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="34"/>
-      <c r="G23" s="37"/>
-      <c r="H23" s="37"/>
-      <c r="I23" s="37"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
-      <c r="L23" s="34"/>
-      <c r="M23" s="37"/>
-      <c r="N23" s="34"/>
-      <c r="O23" s="34"/>
-      <c r="P23" s="38"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="25"/>
+      <c r="D23" s="26"/>
+      <c r="E23" s="27"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="28"/>
+      <c r="I23" s="28"/>
+      <c r="M23" s="28"/>
+      <c r="P23" s="29"/>
     </row>
     <row r="24" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="32"/>
-      <c r="B24" s="33"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="34"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="37"/>
-      <c r="I24" s="37"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="34"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="34"/>
-      <c r="O24" s="34"/>
-      <c r="P24" s="38"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="25"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="27"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="M24" s="28"/>
+      <c r="P24" s="29"/>
     </row>
     <row r="25" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="32"/>
-      <c r="B25" s="33"/>
-      <c r="C25" s="34"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-      <c r="I25" s="37"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
-      <c r="L25" s="34"/>
-      <c r="M25" s="37"/>
-      <c r="N25" s="34"/>
-      <c r="O25" s="34"/>
-      <c r="P25" s="38"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="25"/>
+      <c r="D25" s="26"/>
+      <c r="E25" s="27"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="28"/>
+      <c r="I25" s="28"/>
+      <c r="M25" s="28"/>
+      <c r="P25" s="29"/>
     </row>
     <row r="26" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="32"/>
-      <c r="B26" s="33"/>
-      <c r="C26" s="34"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="34"/>
-      <c r="G26" s="37"/>
-      <c r="H26" s="37"/>
-      <c r="I26" s="37"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
-      <c r="L26" s="34"/>
-      <c r="M26" s="37"/>
-      <c r="N26" s="34"/>
-      <c r="O26" s="34"/>
-      <c r="P26" s="38"/>
+      <c r="A26" s="24"/>
+      <c r="B26" s="25"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="27"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="28"/>
+      <c r="I26" s="28"/>
+      <c r="M26" s="28"/>
+      <c r="P26" s="29"/>
     </row>
     <row r="27" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="32"/>
-      <c r="B27" s="33"/>
-      <c r="C27" s="34"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="34"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="37"/>
-      <c r="I27" s="37"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
-      <c r="L27" s="34"/>
-      <c r="M27" s="37"/>
-      <c r="N27" s="34"/>
-      <c r="O27" s="34"/>
-      <c r="P27" s="38"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="25"/>
+      <c r="D27" s="26"/>
+      <c r="E27" s="27"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
+      <c r="M27" s="28"/>
+      <c r="P27" s="29"/>
     </row>
     <row r="28" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="32"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="34"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="37"/>
-      <c r="H28" s="37"/>
-      <c r="I28" s="37"/>
-      <c r="J28" s="34"/>
-      <c r="K28" s="34"/>
-      <c r="L28" s="34"/>
-      <c r="M28" s="37"/>
-      <c r="N28" s="34"/>
-      <c r="O28" s="34"/>
-      <c r="P28" s="38"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="25"/>
+      <c r="D28" s="26"/>
+      <c r="E28" s="27"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="28"/>
+      <c r="I28" s="28"/>
+      <c r="M28" s="28"/>
+      <c r="P28" s="29"/>
     </row>
     <row r="29" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="32"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="36"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="37"/>
-      <c r="H29" s="37"/>
-      <c r="I29" s="37"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="37"/>
-      <c r="N29" s="34"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="38"/>
+      <c r="A29" s="24"/>
+      <c r="B29" s="25"/>
+      <c r="D29" s="26"/>
+      <c r="E29" s="27"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
+      <c r="M29" s="28"/>
+      <c r="P29" s="29"/>
     </row>
     <row r="30" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="32"/>
-      <c r="B30" s="33"/>
-      <c r="C30" s="34"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="34"/>
-      <c r="G30" s="37"/>
-      <c r="H30" s="37"/>
-      <c r="I30" s="37"/>
-      <c r="J30" s="34"/>
-      <c r="K30" s="34"/>
-      <c r="L30" s="34"/>
-      <c r="M30" s="37"/>
-      <c r="N30" s="34"/>
-      <c r="O30" s="34"/>
-      <c r="P30" s="38"/>
+      <c r="A30" s="24"/>
+      <c r="B30" s="25"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="27"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="M30" s="28"/>
+      <c r="P30" s="29"/>
     </row>
     <row r="31" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="32"/>
-      <c r="B31" s="33"/>
-      <c r="C31" s="34"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="36"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="37"/>
-      <c r="H31" s="37"/>
-      <c r="I31" s="37"/>
-      <c r="J31" s="34"/>
-      <c r="K31" s="34"/>
-      <c r="L31" s="34"/>
-      <c r="M31" s="37"/>
-      <c r="N31" s="34"/>
-      <c r="O31" s="34"/>
-      <c r="P31" s="38"/>
+      <c r="A31" s="24"/>
+      <c r="B31" s="25"/>
+      <c r="D31" s="26"/>
+      <c r="E31" s="27"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="M31" s="28"/>
+      <c r="P31" s="29"/>
     </row>
     <row r="32" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="32"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="34"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="37"/>
-      <c r="J32" s="34"/>
-      <c r="K32" s="34"/>
-      <c r="L32" s="34"/>
-      <c r="M32" s="37"/>
-      <c r="N32" s="34"/>
-      <c r="O32" s="34"/>
-      <c r="P32" s="38"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="25"/>
+      <c r="D32" s="26"/>
+      <c r="E32" s="27"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="M32" s="28"/>
+      <c r="P32" s="29"/>
     </row>
     <row r="33" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="32"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="34"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="34"/>
-      <c r="G33" s="37"/>
-      <c r="H33" s="37"/>
-      <c r="I33" s="37"/>
-      <c r="J33" s="34"/>
-      <c r="K33" s="34"/>
-      <c r="L33" s="34"/>
-      <c r="M33" s="37"/>
-      <c r="N33" s="34"/>
-      <c r="O33" s="34"/>
-      <c r="P33" s="38"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="25"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="27"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="M33" s="28"/>
+      <c r="P33" s="29"/>
     </row>
     <row r="34" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="32"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="34"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="37"/>
-      <c r="H34" s="37"/>
-      <c r="I34" s="37"/>
-      <c r="J34" s="34"/>
-      <c r="K34" s="34"/>
-      <c r="L34" s="34"/>
-      <c r="M34" s="37"/>
-      <c r="N34" s="34"/>
-      <c r="O34" s="34"/>
-      <c r="P34" s="38"/>
+      <c r="A34" s="24"/>
+      <c r="B34" s="25"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="27"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="28"/>
+      <c r="I34" s="28"/>
+      <c r="M34" s="28"/>
+      <c r="P34" s="29"/>
     </row>
     <row r="35" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="32"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="34"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="34"/>
-      <c r="G35" s="37"/>
-      <c r="H35" s="37"/>
-      <c r="I35" s="37"/>
-      <c r="J35" s="34"/>
-      <c r="K35" s="34"/>
-      <c r="L35" s="34"/>
-      <c r="M35" s="37"/>
-      <c r="N35" s="34"/>
-      <c r="O35" s="34"/>
-      <c r="P35" s="38"/>
+      <c r="A35" s="24"/>
+      <c r="B35" s="25"/>
+      <c r="D35" s="26"/>
+      <c r="E35" s="27"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="M35" s="28"/>
+      <c r="P35" s="29"/>
     </row>
     <row r="36" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="32"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="34"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="34"/>
-      <c r="G36" s="37"/>
-      <c r="H36" s="37"/>
-      <c r="I36" s="37"/>
-      <c r="J36" s="34"/>
-      <c r="K36" s="34"/>
-      <c r="L36" s="34"/>
-      <c r="M36" s="37"/>
-      <c r="N36" s="34"/>
-      <c r="O36" s="34"/>
-      <c r="P36" s="38"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="25"/>
+      <c r="D36" s="26"/>
+      <c r="E36" s="27"/>
+      <c r="G36" s="28"/>
+      <c r="H36" s="28"/>
+      <c r="I36" s="28"/>
+      <c r="M36" s="28"/>
+      <c r="P36" s="29"/>
     </row>
     <row r="37" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="32"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="34"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="34"/>
-      <c r="G37" s="37"/>
-      <c r="H37" s="37"/>
-      <c r="I37" s="37"/>
-      <c r="J37" s="34"/>
-      <c r="K37" s="34"/>
-      <c r="L37" s="34"/>
-      <c r="M37" s="37"/>
-      <c r="N37" s="34"/>
-      <c r="O37" s="34"/>
-      <c r="P37" s="38"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="25"/>
+      <c r="D37" s="26"/>
+      <c r="E37" s="27"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="28"/>
+      <c r="I37" s="28"/>
+      <c r="M37" s="28"/>
+      <c r="P37" s="29"/>
     </row>
     <row r="38" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="32"/>
-      <c r="B38" s="33"/>
-      <c r="C38" s="34"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="36"/>
-      <c r="F38" s="34"/>
-      <c r="G38" s="37"/>
-      <c r="H38" s="37"/>
-      <c r="I38" s="37"/>
-      <c r="J38" s="34"/>
-      <c r="K38" s="34"/>
-      <c r="L38" s="34"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="34"/>
-      <c r="O38" s="34"/>
-      <c r="P38" s="38"/>
+      <c r="A38" s="24"/>
+      <c r="B38" s="25"/>
+      <c r="D38" s="26"/>
+      <c r="E38" s="27"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="28"/>
+      <c r="I38" s="28"/>
+      <c r="M38" s="28"/>
+      <c r="P38" s="29"/>
     </row>
     <row r="39" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="32"/>
-      <c r="B39" s="33"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="36"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="37"/>
-      <c r="I39" s="37"/>
-      <c r="J39" s="34"/>
-      <c r="K39" s="34"/>
-      <c r="L39" s="34"/>
-      <c r="M39" s="37"/>
-      <c r="N39" s="34"/>
-      <c r="O39" s="34"/>
-      <c r="P39" s="38"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="25"/>
+      <c r="D39" s="26"/>
+      <c r="E39" s="27"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="28"/>
+      <c r="I39" s="28"/>
+      <c r="M39" s="28"/>
+      <c r="P39" s="29"/>
     </row>
     <row r="40" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="32"/>
-      <c r="B40" s="33"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="36"/>
-      <c r="F40" s="34"/>
-      <c r="G40" s="37"/>
-      <c r="H40" s="37"/>
-      <c r="I40" s="37"/>
-      <c r="J40" s="34"/>
-      <c r="K40" s="34"/>
-      <c r="L40" s="34"/>
-      <c r="M40" s="37"/>
-      <c r="N40" s="34"/>
-      <c r="O40" s="34"/>
-      <c r="P40" s="38"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="25"/>
+      <c r="D40" s="26"/>
+      <c r="E40" s="27"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="28"/>
+      <c r="I40" s="28"/>
+      <c r="M40" s="28"/>
+      <c r="P40" s="29"/>
     </row>
     <row r="41" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="32"/>
-      <c r="B41" s="33"/>
-      <c r="C41" s="34"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="36"/>
-      <c r="F41" s="34"/>
-      <c r="G41" s="37"/>
-      <c r="H41" s="37"/>
-      <c r="I41" s="37"/>
-      <c r="J41" s="34"/>
-      <c r="K41" s="34"/>
-      <c r="L41" s="34"/>
-      <c r="M41" s="37"/>
-      <c r="N41" s="34"/>
-      <c r="O41" s="34"/>
-      <c r="P41" s="38"/>
+      <c r="A41" s="24"/>
+      <c r="B41" s="25"/>
+      <c r="D41" s="26"/>
+      <c r="E41" s="27"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="28"/>
+      <c r="I41" s="28"/>
+      <c r="M41" s="28"/>
+      <c r="P41" s="29"/>
     </row>
     <row r="42" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="32"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="34"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="36"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="37"/>
-      <c r="H42" s="37"/>
-      <c r="I42" s="37"/>
-      <c r="J42" s="34"/>
-      <c r="K42" s="34"/>
-      <c r="L42" s="34"/>
-      <c r="M42" s="37"/>
-      <c r="N42" s="34"/>
-      <c r="O42" s="34"/>
-      <c r="P42" s="38"/>
+      <c r="A42" s="24"/>
+      <c r="B42" s="25"/>
+      <c r="D42" s="26"/>
+      <c r="E42" s="27"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="28"/>
+      <c r="I42" s="28"/>
+      <c r="M42" s="28"/>
+      <c r="P42" s="29"/>
     </row>
     <row r="43" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="32"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="34"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="36"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="37"/>
-      <c r="H43" s="37"/>
-      <c r="I43" s="37"/>
-      <c r="J43" s="34"/>
-      <c r="K43" s="34"/>
-      <c r="L43" s="34"/>
-      <c r="M43" s="37"/>
-      <c r="N43" s="34"/>
-      <c r="O43" s="34"/>
-      <c r="P43" s="38"/>
+      <c r="A43" s="24"/>
+      <c r="B43" s="25"/>
+      <c r="D43" s="26"/>
+      <c r="E43" s="27"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="28"/>
+      <c r="I43" s="28"/>
+      <c r="M43" s="28"/>
+      <c r="P43" s="29"/>
     </row>
     <row r="44" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="32"/>
-      <c r="B44" s="33"/>
-      <c r="C44" s="34"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="36"/>
-      <c r="F44" s="34"/>
-      <c r="G44" s="37"/>
-      <c r="H44" s="37"/>
-      <c r="I44" s="37"/>
-      <c r="J44" s="34"/>
-      <c r="K44" s="34"/>
-      <c r="L44" s="34"/>
-      <c r="M44" s="37"/>
-      <c r="N44" s="34"/>
-      <c r="O44" s="34"/>
-      <c r="P44" s="38"/>
+      <c r="A44" s="24"/>
+      <c r="B44" s="25"/>
+      <c r="D44" s="26"/>
+      <c r="E44" s="27"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="28"/>
+      <c r="I44" s="28"/>
+      <c r="M44" s="28"/>
+      <c r="P44" s="29"/>
     </row>
     <row r="45" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="32"/>
-      <c r="B45" s="33"/>
-      <c r="C45" s="34"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="36"/>
-      <c r="F45" s="34"/>
-      <c r="G45" s="37"/>
-      <c r="H45" s="37"/>
-      <c r="I45" s="37"/>
-      <c r="J45" s="34"/>
-      <c r="K45" s="34"/>
-      <c r="L45" s="34"/>
-      <c r="M45" s="37"/>
-      <c r="N45" s="34"/>
-      <c r="O45" s="34"/>
-      <c r="P45" s="38"/>
+      <c r="A45" s="24"/>
+      <c r="B45" s="25"/>
+      <c r="D45" s="26"/>
+      <c r="E45" s="27"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="28"/>
+      <c r="I45" s="28"/>
+      <c r="M45" s="28"/>
+      <c r="P45" s="29"/>
     </row>
     <row r="46" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="32"/>
-      <c r="B46" s="33"/>
-      <c r="C46" s="34"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="36"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="37"/>
-      <c r="H46" s="37"/>
-      <c r="I46" s="37"/>
-      <c r="J46" s="34"/>
-      <c r="K46" s="34"/>
-      <c r="L46" s="34"/>
-      <c r="M46" s="37"/>
-      <c r="N46" s="34"/>
-      <c r="O46" s="34"/>
-      <c r="P46" s="38"/>
+      <c r="A46" s="24"/>
+      <c r="B46" s="25"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="27"/>
+      <c r="G46" s="28"/>
+      <c r="H46" s="28"/>
+      <c r="I46" s="28"/>
+      <c r="M46" s="28"/>
+      <c r="P46" s="29"/>
     </row>
     <row r="47" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="32"/>
-      <c r="B47" s="33"/>
-      <c r="C47" s="34"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="36"/>
-      <c r="F47" s="34"/>
-      <c r="G47" s="37"/>
-      <c r="H47" s="37"/>
-      <c r="I47" s="37"/>
-      <c r="J47" s="34"/>
-      <c r="K47" s="34"/>
-      <c r="L47" s="34"/>
-      <c r="M47" s="37"/>
-      <c r="N47" s="34"/>
-      <c r="O47" s="34"/>
-      <c r="P47" s="38"/>
+      <c r="A47" s="24"/>
+      <c r="B47" s="25"/>
+      <c r="D47" s="26"/>
+      <c r="E47" s="27"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="28"/>
+      <c r="I47" s="28"/>
+      <c r="M47" s="28"/>
+      <c r="P47" s="29"/>
     </row>
     <row r="48" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="32"/>
-      <c r="B48" s="33"/>
-      <c r="C48" s="34"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="36"/>
-      <c r="F48" s="34"/>
-      <c r="G48" s="37"/>
-      <c r="H48" s="37"/>
-      <c r="I48" s="37"/>
-      <c r="J48" s="34"/>
-      <c r="K48" s="34"/>
-      <c r="L48" s="34"/>
-      <c r="M48" s="37"/>
-      <c r="N48" s="34"/>
-      <c r="O48" s="34"/>
-      <c r="P48" s="38"/>
+      <c r="A48" s="24"/>
+      <c r="B48" s="25"/>
+      <c r="D48" s="26"/>
+      <c r="E48" s="27"/>
+      <c r="G48" s="28"/>
+      <c r="H48" s="28"/>
+      <c r="I48" s="28"/>
+      <c r="M48" s="28"/>
+      <c r="P48" s="29"/>
     </row>
     <row r="49" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="32"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="34"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="36"/>
-      <c r="F49" s="34"/>
-      <c r="G49" s="37"/>
-      <c r="H49" s="37"/>
-      <c r="I49" s="37"/>
-      <c r="J49" s="34"/>
-      <c r="K49" s="34"/>
-      <c r="L49" s="34"/>
-      <c r="M49" s="37"/>
-      <c r="N49" s="34"/>
-      <c r="O49" s="34"/>
-      <c r="P49" s="38"/>
+      <c r="A49" s="24"/>
+      <c r="B49" s="25"/>
+      <c r="D49" s="26"/>
+      <c r="E49" s="27"/>
+      <c r="G49" s="28"/>
+      <c r="H49" s="28"/>
+      <c r="I49" s="28"/>
+      <c r="M49" s="28"/>
+      <c r="P49" s="29"/>
     </row>
     <row r="50" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="32"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="34"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="36"/>
-      <c r="F50" s="34"/>
-      <c r="G50" s="37"/>
-      <c r="H50" s="37"/>
-      <c r="I50" s="37"/>
-      <c r="J50" s="34"/>
-      <c r="K50" s="34"/>
-      <c r="L50" s="34"/>
-      <c r="M50" s="37"/>
-      <c r="N50" s="34"/>
-      <c r="O50" s="34"/>
-      <c r="P50" s="38"/>
+      <c r="A50" s="24"/>
+      <c r="B50" s="25"/>
+      <c r="D50" s="26"/>
+      <c r="E50" s="27"/>
+      <c r="G50" s="28"/>
+      <c r="H50" s="28"/>
+      <c r="I50" s="28"/>
+      <c r="M50" s="28"/>
+      <c r="P50" s="29"/>
     </row>
     <row r="51" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="32"/>
-      <c r="B51" s="33"/>
-      <c r="C51" s="34"/>
-      <c r="D51" s="35"/>
-      <c r="E51" s="36"/>
-      <c r="F51" s="34"/>
-      <c r="G51" s="37"/>
-      <c r="H51" s="37"/>
-      <c r="I51" s="37"/>
-      <c r="J51" s="34"/>
-      <c r="K51" s="34"/>
-      <c r="L51" s="34"/>
-      <c r="M51" s="37"/>
-      <c r="N51" s="34"/>
-      <c r="O51" s="34"/>
-      <c r="P51" s="38"/>
+      <c r="A51" s="24"/>
+      <c r="B51" s="25"/>
+      <c r="D51" s="26"/>
+      <c r="E51" s="27"/>
+      <c r="G51" s="28"/>
+      <c r="H51" s="28"/>
+      <c r="I51" s="28"/>
+      <c r="M51" s="28"/>
+      <c r="P51" s="29"/>
     </row>
     <row r="52" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="32"/>
-      <c r="B52" s="33"/>
-      <c r="C52" s="34"/>
-      <c r="D52" s="35"/>
-      <c r="E52" s="36"/>
-      <c r="F52" s="34"/>
-      <c r="G52" s="37"/>
-      <c r="H52" s="37"/>
-      <c r="I52" s="37"/>
-      <c r="J52" s="34"/>
-      <c r="K52" s="34"/>
-      <c r="L52" s="34"/>
-      <c r="M52" s="37"/>
-      <c r="N52" s="34"/>
-      <c r="O52" s="34"/>
-      <c r="P52" s="38"/>
+      <c r="A52" s="24"/>
+      <c r="B52" s="25"/>
+      <c r="D52" s="26"/>
+      <c r="E52" s="27"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="28"/>
+      <c r="I52" s="28"/>
+      <c r="M52" s="28"/>
+      <c r="P52" s="29"/>
     </row>
     <row r="53" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="32"/>
-      <c r="B53" s="33"/>
-      <c r="C53" s="34"/>
-      <c r="D53" s="35"/>
-      <c r="E53" s="36"/>
-      <c r="F53" s="34"/>
-      <c r="G53" s="37"/>
-      <c r="H53" s="37"/>
-      <c r="I53" s="37"/>
-      <c r="J53" s="34"/>
-      <c r="K53" s="34"/>
-      <c r="L53" s="34"/>
-      <c r="M53" s="37"/>
-      <c r="N53" s="34"/>
-      <c r="O53" s="34"/>
-      <c r="P53" s="38"/>
+      <c r="A53" s="24"/>
+      <c r="B53" s="25"/>
+      <c r="D53" s="26"/>
+      <c r="E53" s="27"/>
+      <c r="G53" s="28"/>
+      <c r="H53" s="28"/>
+      <c r="I53" s="28"/>
+      <c r="M53" s="28"/>
+      <c r="P53" s="29"/>
     </row>
     <row r="54" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="32"/>
-      <c r="B54" s="33"/>
-      <c r="C54" s="34"/>
-      <c r="D54" s="35"/>
-      <c r="E54" s="36"/>
-      <c r="F54" s="34"/>
-      <c r="G54" s="37"/>
-      <c r="H54" s="37"/>
-      <c r="I54" s="37"/>
-      <c r="J54" s="34"/>
-      <c r="K54" s="34"/>
-      <c r="L54" s="34"/>
-      <c r="M54" s="37"/>
-      <c r="N54" s="34"/>
-      <c r="O54" s="34"/>
-      <c r="P54" s="38"/>
+      <c r="A54" s="24"/>
+      <c r="B54" s="25"/>
+      <c r="D54" s="26"/>
+      <c r="E54" s="27"/>
+      <c r="G54" s="28"/>
+      <c r="H54" s="28"/>
+      <c r="I54" s="28"/>
+      <c r="M54" s="28"/>
+      <c r="P54" s="29"/>
     </row>
     <row r="55" spans="1:16" s="2" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="32"/>
-      <c r="B55" s="33"/>
-      <c r="C55" s="34"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="36"/>
-      <c r="F55" s="34"/>
-      <c r="G55" s="37"/>
-      <c r="H55" s="37"/>
-      <c r="I55" s="37"/>
-      <c r="J55" s="34"/>
-      <c r="K55" s="34"/>
-      <c r="L55" s="34"/>
-      <c r="M55" s="37"/>
-      <c r="N55" s="34"/>
-      <c r="O55" s="34"/>
-      <c r="P55" s="38"/>
+      <c r="A55" s="24"/>
+      <c r="B55" s="25"/>
+      <c r="D55" s="26"/>
+      <c r="E55" s="27"/>
+      <c r="G55" s="28"/>
+      <c r="H55" s="28"/>
+      <c r="I55" s="28"/>
+      <c r="M55" s="28"/>
+      <c r="P55" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2053,77 +1700,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">2015-09-03T14:30:00+00:00</_DCDateModified>
-    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
-    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Einarbeitung Ergebnisse WS in 03/2015</_Revision>
-    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-</file>
-
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="6" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="3d4e64bebabe581e87caa1b5e2dea503">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="85eee936267896b8f15e0fd2c7a0c6ca" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -2335,41 +1911,78 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A250377D-DB34-4D72-A19F-2F73A6252A0A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB696076-B3D6-4AD0-BF4E-1EF9EBF80159}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2333D3E7-47AC-4551-8F02-793828071345}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">2015-09-03T14:30:00+00:00</_DCDateModified>
+    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
+    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Einarbeitung Ergebnisse WS in 03/2015</_Revision>
+    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02C699D6-D292-4158-BA61-B30266890DD0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810CFAC6-F050-4FE9-8D40-27B8B016658F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2386,4 +1999,38 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02C699D6-D292-4158-BA61-B30266890DD0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2333D3E7-47AC-4551-8F02-793828071345}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB696076-B3D6-4AD0-BF4E-1EF9EBF80159}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A250377D-DB34-4D72-A19F-2F73A6252A0A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Sskz, Sskx: Modify export pdf (#2319)
Co-authored-by: Marius Heine <m.heine@geprog.com>
</commit_message>
<xml_diff>
--- a/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskx_vorlage.xlsx
+++ b/java/bundles/org.eclipse.set.feature/rootdir/data/export/excel/sskx_vorlage.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\SET\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws_intern\planpro\repos\set\java\bundles\org.eclipse.set.feature\rootdir\data\export\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB8F5BD7-5BA9-43A1-97ED-3E489B87791E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35DCC0E-189D-4A23-A21F-AFF97B9D742F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8595" yWindow="2475" windowWidth="28800" windowHeight="15345" tabRatio="501" xr2:uid="{5D844E15-32D4-4E4F-AD6A-36EA8900B557}"/>
+    <workbookView xWindow="630" yWindow="3075" windowWidth="27210" windowHeight="15060" tabRatio="501" xr2:uid="{5D844E15-32D4-4E4F-AD6A-36EA8900B557}"/>
   </bookViews>
   <sheets>
     <sheet name="Sskx_Beispielbefüllung" sheetId="2" r:id="rId1"/>
@@ -1693,13 +1693,84 @@
     <mergeCell ref="N2:O2"/>
     <mergeCell ref="J3:K3"/>
   </mergeCells>
-  <pageMargins left="0.78740157480314965" right="0.78740157480314965" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageMargins left="0.78740157480314965" right="0.39370078740157483" top="0.19685039370078741" bottom="0.59055118110236227" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="8" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">2015-09-03T14:30:00+00:00</_DCDateModified>
+    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
+    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Einarbeitung Ergebnisse WS in 03/2015</_Revision>
+    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E758A0F93049BE4CAD441F10C0D8186D" ma:contentTypeVersion="6" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="3d4e64bebabe581e87caa1b5e2dea503">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="576ce185-3b2e-4f75-8b7c-efeb82226bea" xmlns:ns3="http://schemas.microsoft.com/sharepoint/v3/fields" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="85eee936267896b8f15e0fd2c7a0c6ca" ns2:_="" ns3:_="">
     <xsd:import namespace="576ce185-3b2e-4f75-8b7c-efeb82226bea"/>
@@ -1911,78 +1982,41 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<LongProperties xmlns="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A250377D-DB34-4D72-A19F-2F73A6252A0A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB696076-B3D6-4AD0-BF4E-1EF9EBF80159}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Version xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <_DCDateModified xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">2015-09-03T14:30:00+00:00</_DCDateModified>
-    <_Status xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Nicht begonnen</_Status>
-    <_Revision xmlns="http://schemas.microsoft.com/sharepoint/v3/fields">Einarbeitung Ergebnisse WS in 03/2015</_Revision>
-    <_DCDateCreated xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2333D3E7-47AC-4551-8F02-793828071345}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02C699D6-D292-4158-BA61-B30266890DD0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{810CFAC6-F050-4FE9-8D40-27B8B016658F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1999,38 +2033,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{02C699D6-D292-4158-BA61-B30266890DD0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/longProperties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2333D3E7-47AC-4551-8F02-793828071345}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DB696076-B3D6-4AD0-BF4E-1EF9EBF80159}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A250377D-DB34-4D72-A19F-2F73A6252A0A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>